<commit_message>
daily-jobs: biostat SM/AD scrape for 2026-05-11
</commit_message>
<xml_diff>
--- a/daily-jobs/manual-check-2026-05-11.xlsx
+++ b/daily-jobs/manual-check-2026-05-11.xlsx
@@ -391,7 +391,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1447,7 +1447,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">scanned=0 title_hits=0 in_window=0 (0.1s)</t>
+          <t xml:space="preserve">scanned=0 title_hits=0 in_24h=0 (0.1s)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1767,7 +1767,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">scanned=0 title_hits=0 in_window=0 (0.1s)</t>
+          <t xml:space="preserve">scanned=0 title_hits=0 in_24h=0 (0.1s)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1831,7 +1831,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">scanned=0 title_hits=0 in_window=0 (0.1s)</t>
+          <t xml:space="preserve">scanned=0 title_hits=0 in_24h=0 (0.1s)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2023,7 +2023,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2119,7 +2119,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2567,7 +2567,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 404 Not Found</t>
+          <t xml:space="preserve">no diagnostic</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">

</xml_diff>